<commit_message>
Align integrated journal and downloads with latest 28 October snapshot; archive Kraken capture
</commit_message>
<xml_diff>
--- a/downloads/crypto-journal-2026-10-28.xlsx
+++ b/downloads/crypto-journal-2026-10-28.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="1" r:id="Ra7547de9fd2b4efe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="1" r:id="R336dd98823e94570"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -346,7 +346,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Stand 2026-10-28; Kraken Spot in USDT; technische Marken: berechnete Tagespivots.</x:v>
+        <x:v>Stand 2026-10-28; Binance Spot in USDT; technische Marken: berechnete Tagespivots.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="40" customHeight="1">
@@ -401,40 +401,40 @@
         <x:v>BTC</x:v>
       </x:c>
       <x:c r="C6" s="11" t="n">
-        <x:v>81549.3</x:v>
+        <x:v>80663.78</x:v>
       </x:c>
       <x:c r="D6" s="4" t="str">
-        <x:v>Unter SMA20 (81.948,2); über Tagespivot 80.579,3</x:v>
+        <x:v>Tieferes Hoch / tieferes Tief</x:v>
       </x:c>
       <x:c r="E6" s="4" t="str">
-        <x:v>S1 79.858,6 / S2 78.793,5</x:v>
+        <x:v>S1 79.843,85 / S2 78.777,92</x:v>
       </x:c>
       <x:c r="F6" s="4" t="str">
-        <x:v>R1 81.644,4 / R2 82.365,1</x:v>
+        <x:v>R1 81.637,85 / R2 82.365,92</x:v>
       </x:c>
       <x:c r="G6" s="4" t="str">
-        <x:v>79.858,6–80.579,3 (Pivot-Rücklauf; Bestätigung abwarten)</x:v>
+        <x:v>79.843,85–80.571,92</x:v>
       </x:c>
       <x:c r="H6" s="4" t="str">
-        <x:v>81.644,4–82.365,1 (nur bei Ablehnung)</x:v>
+        <x:v>81.637,85–82.365,92</x:v>
       </x:c>
       <x:c r="I6" s="11" t="n">
-        <x:v>81644.36666666668</x:v>
+        <x:v>81637.84666666668</x:v>
       </x:c>
       <x:c r="J6" s="11" t="n">
-        <x:v>79858.56666666668</x:v>
+        <x:v>79843.84666666668</x:v>
       </x:c>
       <x:c r="K6" s="4" t="str">
-        <x:v>Oberseite R1/R2: 81.644,4 / 82.365,1; Unterseite S1/S2: 79.858,6 / 78.793,5</x:v>
+        <x:v>Long R1/R2 81.637,85 / 82.365,92; Short Pivot/S1 80.571,92 / 79.843,85</x:v>
       </x:c>
       <x:c r="L6" s="4" t="str">
-        <x:v>Keine aktuelle Liquidationsquelle; alte Heatmap: 03.10.2026</x:v>
+        <x:v>Keine Heatmap</x:v>
       </x:c>
       <x:c r="M6" s="10" t="str">
         <x:v>Nicht verfügbar</x:v>
       </x:c>
       <x:c r="N6" s="10" t="n">
-        <x:v>0.0077319842419270035</x:v>
+        <x:v>-0.0030403003246703975</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="100" customHeight="1">
@@ -445,45 +445,45 @@
         <x:v>XRP</x:v>
       </x:c>
       <x:c r="C7" s="9" t="n">
-        <x:v>1.32948</x:v>
+        <x:v>1.3155</x:v>
       </x:c>
       <x:c r="D7" s="4" t="str">
-        <x:v>Unter SMA20 (1,3362); über Tagespivot 1,3199</x:v>
+        <x:v>Tieferes Hoch / tieferes Tief</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
-        <x:v>S1 1,3032 / S2 1,2748</x:v>
+        <x:v>S1 1,30333 / S2 1,27537</x:v>
       </x:c>
       <x:c r="F7" s="4" t="str">
-        <x:v>R1 1,3483 / R2 1,3649</x:v>
+        <x:v>R1 1,34693 / R2 1,36257</x:v>
       </x:c>
       <x:c r="G7" s="4" t="str">
-        <x:v>1,3032–1,3199 (Pivot-Rücklauf; Bestätigung abwarten)</x:v>
+        <x:v>1,30333–1,31897</x:v>
       </x:c>
       <x:c r="H7" s="4" t="str">
-        <x:v>1,3483–1,3649 (nur bei Ablehnung)</x:v>
+        <x:v>1,34693–1,36257</x:v>
       </x:c>
       <x:c r="I7" s="9" t="n">
-        <x:v>1.3482733333333332</x:v>
+        <x:v>1.3469333333333333</x:v>
       </x:c>
       <x:c r="J7" s="9" t="n">
-        <x:v>1.303243333333333</x:v>
+        <x:v>1.3033333333333332</x:v>
       </x:c>
       <x:c r="K7" s="4" t="str">
-        <x:v>Oberseite R1/R2: 1,3483 / 1,3649; Unterseite S1/S2: 1,3032 / 1,2748</x:v>
+        <x:v>Long R1/R2 1,34693 / 1,36257; Short Pivot/S1 1,31897 / 1,30333</x:v>
       </x:c>
       <x:c r="L7" s="4" t="str">
-        <x:v>Keine aktuelle Liquidationsquelle; alte Heatmap: 03.10.2026</x:v>
+        <x:v>Keine Heatmap</x:v>
       </x:c>
       <x:c r="M7" s="10" t="str">
         <x:v>Nicht verfügbar</x:v>
       </x:c>
       <x:c r="N7" s="10" t="n">
-        <x:v>-0.0016220600162205612</x:v>
+        <x:v>-0.011868098850747466</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="12" t="str">
-        <x:v>Kraken Spot BTC/USDT und XRP/USDT. Abruf 28.10.2026, 11:25 Uhr Europe/Berlin; Börsenzeit bestätigt. Veränderung: aktueller letzter Handel gegen Kraken-Schlusskurs des 27.10.2026 (UTC), nicht gegen den älteren Journal-Screenshot. Trend: Kurs gegen SMA20 der abgeschlossenen UTC-Tage. Klassische Tagespivots: P=(Vortagshoch+Vortagstief+Vortagsschluss)/3; S1=2P-H, R1=2P-L, S2=P-(H-L), R2=P+(H-L). Zonen und Ziele sind daraus abgeleitete Szenarien; keine unabhängig bestätigten Chart-Signale. Aktuelle Liquidations-Heatmap fehlt; Grafikstand 03.10.2026 bleibt separat erhalten.</x:v>
+        <x:v>Binance Spot · 28.10.2026 16:01 Uhr Europe/Berlin; echte Kerzen und Pivot-Szenarien des abgeschlossenen UTC-Vortags. Keine Heatmap.</x:v>
       </x:c>
       <x:c r="B9" s="12"/>
       <x:c r="C9" s="12"/>
@@ -533,10 +533,8 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="12" t="str">
-        <x:v>https://api.kraken.com/0/public/Ticker?pair=XBTUSDT,XRPUSDT
-https://api.kraken.com/0/public/OHLC?pair=XBTUSDT&amp;interval=1440
-https://api.kraken.com/0/public/OHLC?pair=XRPUSDT&amp;interval=1440
-https://api.kraken.com/0/public/Time</x:v>
+        <x:v>https://data-api.binance.vision/api/v3/klines?symbol=BTCUSDT&amp;interval=30m&amp;limit=300
+https://data-api.binance.vision/api/v3/klines?symbol=XRPUSDT&amp;interval=30m&amp;limit=300</x:v>
       </x:c>
       <x:c r="B13" s="12"/>
       <x:c r="C13" s="12"/>
@@ -607,7 +605,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55d28846637d4d61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf61519f2acb4c18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>